<commit_message>
sample file uploaded for bulk question add
</commit_message>
<xml_diff>
--- a/api/public/sample-files/DE_Bulk_Question_Insert_Sample.xlsx
+++ b/api/public/sample-files/DE_Bulk_Question_Insert_Sample.xlsx
@@ -1,42 +1,128 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10308"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/omkarpatole/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59676523-301F-3641-86A8-45DF33785ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E60BA43A-010E-2949-B1C7-49D5099F2CC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="600" windowWidth="24380" windowHeight="14760" xr2:uid="{203A2A3F-3A2B-9944-9130-CC10A0D29E59}"/>
+    <workbookView xWindow="1140" yWindow="600" windowWidth="24460" windowHeight="15400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
+  <si>
+    <r>
+      <t xml:space="preserve">Test Clerical Aptitude
+In a question below a combination of Name and Address is given followed by four such combinations.  You have to find out the combination which is exactly the same as the combination in question section. The (A), (B), (C) or (D) that contains that combination is the answer.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Kokila"/>
+        <family val="2"/>
+      </rPr>
+      <t>4 El Bazry Street, Off 77 St, Cairo, 11431, Egypt</t>
+    </r>
+  </si>
+  <si>
+    <t>4 El Bazry Street, Of 77 St, Cairo, 11431, Egypt</t>
+  </si>
+  <si>
+    <t>4 El Bazry Street, Off 77 St, Kairo, 11431, Egypt</t>
+  </si>
+  <si>
+    <t>4 El Bazrry Street, Off 77 St, Cairo, 11431, Egypt</t>
+  </si>
+  <si>
+    <t>4 El Bazry Street, Off 77 St, Cairo, 11431, Egypt</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Partnership</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pradhan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Private </t>
+  </si>
+  <si>
+    <t>Proprietorship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PMSBY या संज्ञेमधील P हे अक्षर पुढीलपैकी काय दर्शविते ?
+In PMSBY, the letter P refers to ….. </t>
+  </si>
+  <si>
+    <t>चेक, पे ऑर्डर, बँकर्स चेक व डीमांड ड्राफ्ट यांना काढलेल्या तारखेपासून किती दिवसाची वैधता असते ?
+What is the validity period of a Check, Pay Order, Banker's Check, and Demand Draft from the date of issue?</t>
+  </si>
+  <si>
+    <t>180 दिवस 
+180 days</t>
+  </si>
+  <si>
+    <t>90 दिवस
+90 days</t>
+  </si>
+  <si>
+    <t>365 दिवस
+365 days</t>
+  </si>
+  <si>
+    <t>150 दिवस
+150 days</t>
+  </si>
+  <si>
+    <t>प्रोप्रायटर शिप मालकी असणार्‍या व्यक्तीचे संड्री डेटर्स हे आर्थिक पत्रकामध्ये खालीलपैकी कोठे दाखविले जातात ?
+In the financial statements of a proprietorship business, under which section are sundry debtors shown?</t>
+  </si>
+  <si>
+    <t>बँलंस शीटच्या लायबिलिटी बाजुस
+Liability side of Balance Sheet</t>
+  </si>
+  <si>
+    <t>नफा तोटा पत्रकाच्या डेबिट बाजुस
+Debit Side of Profit &amp; Loss Account</t>
+  </si>
+  <si>
+    <t>बँलंस शीटच्या असेट बाजुस
+Asset Side of Balance Sheet</t>
+  </si>
+  <si>
+    <t>नफा तोटा पत्रकाच्या क्रेडीट बाजुस
+Credit Side of Profit &amp; Loss Account</t>
+  </si>
+  <si>
+    <t>sr</t>
+  </si>
   <si>
     <t>q</t>
   </si>
@@ -53,32 +139,67 @@
     <t>q_d</t>
   </si>
   <si>
-    <t>q_e</t>
-  </si>
-  <si>
     <t>sol</t>
-  </si>
-  <si>
-    <t>what is 2 + 2 = ?</t>
-  </si>
-  <si>
-    <t>none</t>
-  </si>
-  <si>
-    <t>C</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$-4000439]0"/>
+  </numFmts>
+  <fonts count="8" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Kokila"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Kokila"/>
+      <family val="2"/>
+    </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Nirmala UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Nirmala UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Mangal"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Mangal"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -89,7 +210,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -97,12 +218,88 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -131,39 +328,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -196,26 +393,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -248,23 +428,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -326,6 +489,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -334,13 +504,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -405,128 +568,196 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36596444-C9B4-564A-8724-C26D463D59C4}">
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="50" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="86.5" style="1" customWidth="1"/>
+    <col min="3" max="6" width="19.83203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="6.6640625" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" ht="50" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="150" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>78</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+    </row>
+    <row r="3" spans="1:7" ht="50" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>79</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="101" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>83</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="126" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>84</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
-        <v>22</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2">
-        <v>4</v>
-      </c>
-      <c r="E2">
-        <v>21</v>
-      </c>
-      <c r="G2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>22</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3">
-        <v>4</v>
-      </c>
-      <c r="E3">
-        <v>21</v>
-      </c>
-      <c r="G3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4">
-        <v>4</v>
-      </c>
-      <c r="E4">
-        <v>21</v>
-      </c>
-      <c r="G4" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.59055118110236227" right="0.19685039370078741" top="0.19685039370078741" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="90" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Cambria"&amp;11&amp;KFF751A INTERNAL</oddHeader>
+    <oddFooter>&amp;C &amp;L&amp;"Cambria"&amp;11&amp;KFF751A INTERNAL</oddFooter>
+  </headerFooter>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<Klassify>
+  <SNO>1</SNO>
+  <KDate>2026-03-11 07:59:44</KDate>
+  <Classification>CONFIDENTIAL</Classification>
+  <Subclassification/>
+  <HostName>CEOPC</HostName>
+  <Domain_User>CEOPC/Admin</Domain_User>
+  <IPAdd>10.11.2.39</IPAdd>
+  <FilePath>D:\temp\Exam and Training 15022026\Recruitement Exams\032026\Blank template QP.xlsx</FilePath>
+  <KID>9CB6541D943D639088127846120999</KID>
+  <UniqueName/>
+  <Suggested/>
+  <Justification/>
+</Klassify>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<Klassify>
+  <SNO>2</SNO>
+  <KDate>2026-03-11 22:00:16</KDate>
+  <Classification>INTERNAL</Classification>
+  <Subclassification/>
+  <HostName>CEOPC</HostName>
+  <Domain_User>CEOPC/Admin</Domain_User>
+  <IPAdd>10.11.2.39</IPAdd>
+  <FilePath>D:\temp\Exam and Training 15022026\Recruitement Exams\032026\Blank template QP.xlsx</FilePath>
+  <KID>9CB6541D943D639088127846120999</KID>
+  <UniqueName/>
+  <Suggested/>
+  <Justification/>
+</Klassify>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7650843E-B649-418D-ACA5-B8F9A46B9BAA}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BFB941D8-C241-4F13-B897-1B98C9B43F30}">
+  <ds:schemaRefs/>
+</ds:datastoreItem>
 </file>
</xml_diff>